<commit_message>
feat: Add PAID ARREAR column to Excel sheets & embed User Guide modal on frontend UI
</commit_message>
<xml_diff>
--- a/templates/DPO_Muzaffarpur_Arrear_Forms.xlsx
+++ b/templates/DPO_Muzaffarpur_Arrear_Forms.xlsx
@@ -63,15 +63,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -191,11 +197,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -240,6 +260,17 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -605,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z24"/>
+  <dimension ref="A1:AA24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -623,6 +654,7 @@
     <col width="7" customWidth="1" min="16" max="16"/>
     <col width="6" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="19"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
     <col width="8" customWidth="1" min="20" max="21"/>
     <col width="7" customWidth="1" min="22" max="22"/>
     <col width="10" customWidth="1" min="23" max="23"/>
@@ -672,14 +704,14 @@
       <c r="P3" s="16" t="n"/>
       <c r="Q3" s="16" t="n"/>
       <c r="R3" s="16" t="n"/>
-      <c r="S3" s="16" t="n"/>
       <c r="T3" s="16" t="n"/>
       <c r="U3" s="16" t="n"/>
       <c r="V3" s="16" t="n"/>
       <c r="W3" s="16" t="n"/>
       <c r="X3" s="16" t="n"/>
       <c r="Y3" s="16" t="n"/>
-      <c r="Z3" s="17" t="n"/>
+      <c r="Z3" s="16" t="n"/>
+      <c r="AA3" s="17" t="n"/>
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -712,14 +744,14 @@
         </is>
       </c>
       <c r="R4" s="16" t="n"/>
-      <c r="S4" s="16" t="n"/>
       <c r="T4" s="16" t="n"/>
       <c r="U4" s="16" t="n"/>
       <c r="V4" s="16" t="n"/>
       <c r="W4" s="16" t="n"/>
       <c r="X4" s="16" t="n"/>
       <c r="Y4" s="16" t="n"/>
-      <c r="Z4" s="17" t="n"/>
+      <c r="Z4" s="16" t="n"/>
+      <c r="AA4" s="17" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
@@ -752,14 +784,14 @@
         </is>
       </c>
       <c r="R5" s="16" t="n"/>
-      <c r="S5" s="16" t="n"/>
       <c r="T5" s="16" t="n"/>
       <c r="U5" s="16" t="n"/>
       <c r="V5" s="16" t="n"/>
       <c r="W5" s="16" t="n"/>
       <c r="X5" s="16" t="n"/>
       <c r="Y5" s="16" t="n"/>
-      <c r="Z5" s="17" t="n"/>
+      <c r="Z5" s="16" t="n"/>
+      <c r="AA5" s="17" t="n"/>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
@@ -797,18 +829,24 @@
       <c r="P6" s="16" t="n"/>
       <c r="Q6" s="16" t="n"/>
       <c r="R6" s="17" t="n"/>
-      <c r="S6" s="6" t="inlineStr">
+      <c r="S6" s="20" t="inlineStr">
+        <is>
+          <t>PAID
+ARREAR</t>
+        </is>
+      </c>
+      <c r="T6" s="21" t="inlineStr">
         <is>
           <t>DIFFERENCE</t>
         </is>
       </c>
-      <c r="T6" s="16" t="n"/>
       <c r="U6" s="16" t="n"/>
       <c r="V6" s="16" t="n"/>
       <c r="W6" s="16" t="n"/>
       <c r="X6" s="16" t="n"/>
       <c r="Y6" s="16" t="n"/>
-      <c r="Z6" s="17" t="n"/>
+      <c r="Z6" s="16" t="n"/>
+      <c r="AA6" s="17" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="19" t="n"/>
@@ -899,44 +937,45 @@
 PAY</t>
         </is>
       </c>
-      <c r="S7" s="6" t="inlineStr">
+      <c r="S7" s="22" t="n"/>
+      <c r="T7" s="6" t="inlineStr">
         <is>
           <t>Basic
 Pay</t>
         </is>
       </c>
-      <c r="T7" s="6" t="inlineStr">
+      <c r="U7" s="6" t="inlineStr">
         <is>
           <t>D.A.</t>
         </is>
       </c>
-      <c r="U7" s="6" t="inlineStr">
+      <c r="V7" s="6" t="inlineStr">
         <is>
           <t>H.R.A.</t>
         </is>
       </c>
-      <c r="V7" s="6" t="inlineStr">
+      <c r="W7" s="6" t="inlineStr">
         <is>
           <t>M.A.</t>
         </is>
       </c>
-      <c r="W7" s="6" t="inlineStr">
+      <c r="X7" s="6" t="inlineStr">
         <is>
           <t>GROSS
 PAY</t>
         </is>
       </c>
-      <c r="X7" s="6" t="inlineStr">
+      <c r="Y7" s="6" t="inlineStr">
         <is>
           <t>NPS</t>
         </is>
       </c>
-      <c r="Y7" s="6" t="inlineStr">
+      <c r="Z7" s="6" t="inlineStr">
         <is>
           <t>GIS</t>
         </is>
       </c>
-      <c r="Z7" s="6" t="inlineStr">
+      <c r="AA7" s="6" t="inlineStr">
         <is>
           <t>NET
 PAY</t>
@@ -962,7 +1001,7 @@
       <c r="P8" s="7" t="n"/>
       <c r="Q8" s="7" t="n"/>
       <c r="R8" s="7" t="n"/>
-      <c r="S8" s="7" t="n"/>
+      <c r="S8" s="23" t="n"/>
       <c r="T8" s="7" t="n"/>
       <c r="U8" s="7" t="n"/>
       <c r="V8" s="7" t="n"/>
@@ -970,6 +1009,7 @@
       <c r="X8" s="7" t="n"/>
       <c r="Y8" s="7" t="n"/>
       <c r="Z8" s="7" t="n"/>
+      <c r="AA8" s="7" t="n"/>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="7" t="n"/>
@@ -990,7 +1030,7 @@
       <c r="P9" s="7" t="n"/>
       <c r="Q9" s="7" t="n"/>
       <c r="R9" s="7" t="n"/>
-      <c r="S9" s="7" t="n"/>
+      <c r="S9" s="23" t="n"/>
       <c r="T9" s="7" t="n"/>
       <c r="U9" s="7" t="n"/>
       <c r="V9" s="7" t="n"/>
@@ -998,6 +1038,7 @@
       <c r="X9" s="7" t="n"/>
       <c r="Y9" s="7" t="n"/>
       <c r="Z9" s="7" t="n"/>
+      <c r="AA9" s="7" t="n"/>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="7" t="n"/>
@@ -1018,7 +1059,7 @@
       <c r="P10" s="7" t="n"/>
       <c r="Q10" s="7" t="n"/>
       <c r="R10" s="7" t="n"/>
-      <c r="S10" s="7" t="n"/>
+      <c r="S10" s="23" t="n"/>
       <c r="T10" s="7" t="n"/>
       <c r="U10" s="7" t="n"/>
       <c r="V10" s="7" t="n"/>
@@ -1026,6 +1067,7 @@
       <c r="X10" s="7" t="n"/>
       <c r="Y10" s="7" t="n"/>
       <c r="Z10" s="7" t="n"/>
+      <c r="AA10" s="7" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="7" t="n"/>
@@ -1046,7 +1088,7 @@
       <c r="P11" s="7" t="n"/>
       <c r="Q11" s="7" t="n"/>
       <c r="R11" s="7" t="n"/>
-      <c r="S11" s="7" t="n"/>
+      <c r="S11" s="23" t="n"/>
       <c r="T11" s="7" t="n"/>
       <c r="U11" s="7" t="n"/>
       <c r="V11" s="7" t="n"/>
@@ -1054,6 +1096,7 @@
       <c r="X11" s="7" t="n"/>
       <c r="Y11" s="7" t="n"/>
       <c r="Z11" s="7" t="n"/>
+      <c r="AA11" s="7" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="7" t="n"/>
@@ -1074,7 +1117,7 @@
       <c r="P12" s="7" t="n"/>
       <c r="Q12" s="7" t="n"/>
       <c r="R12" s="7" t="n"/>
-      <c r="S12" s="7" t="n"/>
+      <c r="S12" s="23" t="n"/>
       <c r="T12" s="7" t="n"/>
       <c r="U12" s="7" t="n"/>
       <c r="V12" s="7" t="n"/>
@@ -1082,6 +1125,7 @@
       <c r="X12" s="7" t="n"/>
       <c r="Y12" s="7" t="n"/>
       <c r="Z12" s="7" t="n"/>
+      <c r="AA12" s="7" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="7" t="n"/>
@@ -1102,7 +1146,7 @@
       <c r="P13" s="7" t="n"/>
       <c r="Q13" s="7" t="n"/>
       <c r="R13" s="7" t="n"/>
-      <c r="S13" s="7" t="n"/>
+      <c r="S13" s="23" t="n"/>
       <c r="T13" s="7" t="n"/>
       <c r="U13" s="7" t="n"/>
       <c r="V13" s="7" t="n"/>
@@ -1110,6 +1154,7 @@
       <c r="X13" s="7" t="n"/>
       <c r="Y13" s="7" t="n"/>
       <c r="Z13" s="7" t="n"/>
+      <c r="AA13" s="7" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="7" t="n"/>
@@ -1130,7 +1175,7 @@
       <c r="P14" s="7" t="n"/>
       <c r="Q14" s="7" t="n"/>
       <c r="R14" s="7" t="n"/>
-      <c r="S14" s="7" t="n"/>
+      <c r="S14" s="23" t="n"/>
       <c r="T14" s="7" t="n"/>
       <c r="U14" s="7" t="n"/>
       <c r="V14" s="7" t="n"/>
@@ -1138,6 +1183,7 @@
       <c r="X14" s="7" t="n"/>
       <c r="Y14" s="7" t="n"/>
       <c r="Z14" s="7" t="n"/>
+      <c r="AA14" s="7" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="7" t="n"/>
@@ -1158,7 +1204,7 @@
       <c r="P15" s="7" t="n"/>
       <c r="Q15" s="7" t="n"/>
       <c r="R15" s="7" t="n"/>
-      <c r="S15" s="7" t="n"/>
+      <c r="S15" s="23" t="n"/>
       <c r="T15" s="7" t="n"/>
       <c r="U15" s="7" t="n"/>
       <c r="V15" s="7" t="n"/>
@@ -1166,6 +1212,7 @@
       <c r="X15" s="7" t="n"/>
       <c r="Y15" s="7" t="n"/>
       <c r="Z15" s="7" t="n"/>
+      <c r="AA15" s="7" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="7" t="n"/>
@@ -1186,7 +1233,7 @@
       <c r="P16" s="7" t="n"/>
       <c r="Q16" s="7" t="n"/>
       <c r="R16" s="7" t="n"/>
-      <c r="S16" s="7" t="n"/>
+      <c r="S16" s="23" t="n"/>
       <c r="T16" s="7" t="n"/>
       <c r="U16" s="7" t="n"/>
       <c r="V16" s="7" t="n"/>
@@ -1194,6 +1241,7 @@
       <c r="X16" s="7" t="n"/>
       <c r="Y16" s="7" t="n"/>
       <c r="Z16" s="7" t="n"/>
+      <c r="AA16" s="7" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="7" t="n"/>
@@ -1214,7 +1262,7 @@
       <c r="P17" s="7" t="n"/>
       <c r="Q17" s="7" t="n"/>
       <c r="R17" s="7" t="n"/>
-      <c r="S17" s="7" t="n"/>
+      <c r="S17" s="23" t="n"/>
       <c r="T17" s="7" t="n"/>
       <c r="U17" s="7" t="n"/>
       <c r="V17" s="7" t="n"/>
@@ -1222,6 +1270,7 @@
       <c r="X17" s="7" t="n"/>
       <c r="Y17" s="7" t="n"/>
       <c r="Z17" s="7" t="n"/>
+      <c r="AA17" s="7" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="7" t="n"/>
@@ -1242,7 +1291,7 @@
       <c r="P18" s="7" t="n"/>
       <c r="Q18" s="7" t="n"/>
       <c r="R18" s="7" t="n"/>
-      <c r="S18" s="7" t="n"/>
+      <c r="S18" s="23" t="n"/>
       <c r="T18" s="7" t="n"/>
       <c r="U18" s="7" t="n"/>
       <c r="V18" s="7" t="n"/>
@@ -1250,6 +1299,7 @@
       <c r="X18" s="7" t="n"/>
       <c r="Y18" s="7" t="n"/>
       <c r="Z18" s="7" t="n"/>
+      <c r="AA18" s="7" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="7" t="n"/>
@@ -1270,7 +1320,7 @@
       <c r="P19" s="7" t="n"/>
       <c r="Q19" s="7" t="n"/>
       <c r="R19" s="7" t="n"/>
-      <c r="S19" s="7" t="n"/>
+      <c r="S19" s="23" t="n"/>
       <c r="T19" s="7" t="n"/>
       <c r="U19" s="7" t="n"/>
       <c r="V19" s="7" t="n"/>
@@ -1278,6 +1328,7 @@
       <c r="X19" s="7" t="n"/>
       <c r="Y19" s="7" t="n"/>
       <c r="Z19" s="7" t="n"/>
+      <c r="AA19" s="7" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="7" t="n"/>
@@ -1298,7 +1349,7 @@
       <c r="P20" s="7" t="n"/>
       <c r="Q20" s="7" t="n"/>
       <c r="R20" s="7" t="n"/>
-      <c r="S20" s="7" t="n"/>
+      <c r="S20" s="23" t="n"/>
       <c r="T20" s="7" t="n"/>
       <c r="U20" s="7" t="n"/>
       <c r="V20" s="7" t="n"/>
@@ -1306,6 +1357,7 @@
       <c r="X20" s="7" t="n"/>
       <c r="Y20" s="7" t="n"/>
       <c r="Z20" s="7" t="n"/>
+      <c r="AA20" s="7" t="n"/>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
@@ -1330,7 +1382,10 @@
       <c r="P21" s="7" t="n"/>
       <c r="Q21" s="7" t="n"/>
       <c r="R21" s="7" t="n"/>
-      <c r="S21" s="7" t="n"/>
+      <c r="S21" s="24">
+        <f>SUM(S8:S20)</f>
+        <v/>
+      </c>
       <c r="T21" s="7" t="n"/>
       <c r="U21" s="7" t="n"/>
       <c r="V21" s="7" t="n"/>
@@ -1338,6 +1393,7 @@
       <c r="X21" s="7" t="n"/>
       <c r="Y21" s="7" t="n"/>
       <c r="Z21" s="7" t="n"/>
+      <c r="AA21" s="7" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="3" t="n"/>
@@ -1362,14 +1418,18 @@
       <c r="P22" s="16" t="n"/>
       <c r="Q22" s="16" t="n"/>
       <c r="R22" s="16" t="n"/>
-      <c r="S22" s="16" t="n"/>
+      <c r="S22" s="22" t="n"/>
       <c r="T22" s="16" t="n"/>
       <c r="U22" s="16" t="n"/>
       <c r="V22" s="16" t="n"/>
       <c r="W22" s="16" t="n"/>
       <c r="X22" s="16" t="n"/>
       <c r="Y22" s="16" t="n"/>
-      <c r="Z22" s="17" t="n"/>
+      <c r="Z22" s="16" t="n"/>
+      <c r="AA22" s="17" t="n"/>
+    </row>
+    <row r="23">
+      <c r="S23" s="22" t="n"/>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
@@ -1382,15 +1442,17 @@
           <t>SIGNATURE AND SEAL OF HEADMASTER</t>
         </is>
       </c>
+      <c r="S24" s="22" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="21">
     <mergeCell ref="R24:Z24"/>
     <mergeCell ref="C6:J6"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="C22:Z22"/>
     <mergeCell ref="A1:Z1"/>
     <mergeCell ref="B6:B7"/>
+    <mergeCell ref="S6:S7"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="S6:Z6"/>
     <mergeCell ref="N3:Z3"/>
@@ -1402,6 +1464,7 @@
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="I4:P4"/>
     <mergeCell ref="Q4:Z4"/>
+    <mergeCell ref="T6:AA6"/>
     <mergeCell ref="A3:M3"/>
     <mergeCell ref="K6:R6"/>
   </mergeCells>
@@ -1416,7 +1479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1430,6 +1493,7 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="13"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="8" customWidth="1" min="16" max="16"/>
@@ -1471,11 +1535,11 @@
       <c r="J3" s="16" t="n"/>
       <c r="K3" s="16" t="n"/>
       <c r="L3" s="16" t="n"/>
-      <c r="M3" s="16" t="n"/>
       <c r="N3" s="16" t="n"/>
       <c r="O3" s="16" t="n"/>
       <c r="P3" s="16" t="n"/>
-      <c r="Q3" s="17" t="n"/>
+      <c r="Q3" s="16" t="n"/>
+      <c r="R3" s="17" t="n"/>
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -1502,11 +1566,11 @@
         </is>
       </c>
       <c r="L4" s="16" t="n"/>
-      <c r="M4" s="16" t="n"/>
       <c r="N4" s="16" t="n"/>
       <c r="O4" s="16" t="n"/>
       <c r="P4" s="16" t="n"/>
-      <c r="Q4" s="17" t="n"/>
+      <c r="Q4" s="16" t="n"/>
+      <c r="R4" s="17" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
@@ -1533,11 +1597,11 @@
         </is>
       </c>
       <c r="L5" s="16" t="n"/>
-      <c r="M5" s="16" t="n"/>
       <c r="N5" s="16" t="n"/>
       <c r="O5" s="16" t="n"/>
       <c r="P5" s="16" t="n"/>
-      <c r="Q5" s="17" t="n"/>
+      <c r="Q5" s="16" t="n"/>
+      <c r="R5" s="17" t="n"/>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
@@ -1569,15 +1633,21 @@
       <c r="J6" s="16" t="n"/>
       <c r="K6" s="16" t="n"/>
       <c r="L6" s="17" t="n"/>
-      <c r="M6" s="6" t="inlineStr">
+      <c r="M6" s="20" t="inlineStr">
+        <is>
+          <t>PAID
+ARREAR</t>
+        </is>
+      </c>
+      <c r="N6" s="21" t="inlineStr">
         <is>
           <t>DIFFERENCE</t>
         </is>
       </c>
-      <c r="N6" s="16" t="n"/>
       <c r="O6" s="16" t="n"/>
       <c r="P6" s="16" t="n"/>
-      <c r="Q6" s="17" t="n"/>
+      <c r="Q6" s="16" t="n"/>
+      <c r="R6" s="17" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="19" t="n"/>
@@ -1638,29 +1708,30 @@
 AMOUNT</t>
         </is>
       </c>
-      <c r="M7" s="6" t="inlineStr">
+      <c r="M7" s="22" t="n"/>
+      <c r="N7" s="6" t="inlineStr">
         <is>
           <t>Basic
 Pay</t>
         </is>
       </c>
-      <c r="N7" s="6" t="inlineStr">
+      <c r="O7" s="6" t="inlineStr">
         <is>
           <t>D.A.</t>
         </is>
       </c>
-      <c r="O7" s="6" t="inlineStr">
+      <c r="P7" s="6" t="inlineStr">
         <is>
           <t>GROSS
 AMOUNT</t>
         </is>
       </c>
-      <c r="P7" s="6" t="inlineStr">
+      <c r="Q7" s="6" t="inlineStr">
         <is>
           <t>NPS</t>
         </is>
       </c>
-      <c r="Q7" s="6" t="inlineStr">
+      <c r="R7" s="6" t="inlineStr">
         <is>
           <t>NET
 AMOUNT</t>
@@ -1680,11 +1751,12 @@
       <c r="J8" s="7" t="n"/>
       <c r="K8" s="7" t="n"/>
       <c r="L8" s="7" t="n"/>
-      <c r="M8" s="7" t="n"/>
+      <c r="M8" s="23" t="n"/>
       <c r="N8" s="7" t="n"/>
       <c r="O8" s="7" t="n"/>
       <c r="P8" s="7" t="n"/>
       <c r="Q8" s="7" t="n"/>
+      <c r="R8" s="7" t="n"/>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="7" t="n"/>
@@ -1699,11 +1771,12 @@
       <c r="J9" s="7" t="n"/>
       <c r="K9" s="7" t="n"/>
       <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7" t="n"/>
+      <c r="M9" s="23" t="n"/>
       <c r="N9" s="7" t="n"/>
       <c r="O9" s="7" t="n"/>
       <c r="P9" s="7" t="n"/>
       <c r="Q9" s="7" t="n"/>
+      <c r="R9" s="7" t="n"/>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="7" t="n"/>
@@ -1718,11 +1791,12 @@
       <c r="J10" s="7" t="n"/>
       <c r="K10" s="7" t="n"/>
       <c r="L10" s="7" t="n"/>
-      <c r="M10" s="7" t="n"/>
+      <c r="M10" s="23" t="n"/>
       <c r="N10" s="7" t="n"/>
       <c r="O10" s="7" t="n"/>
       <c r="P10" s="7" t="n"/>
       <c r="Q10" s="7" t="n"/>
+      <c r="R10" s="7" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="7" t="n"/>
@@ -1737,11 +1811,12 @@
       <c r="J11" s="7" t="n"/>
       <c r="K11" s="7" t="n"/>
       <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7" t="n"/>
+      <c r="M11" s="23" t="n"/>
       <c r="N11" s="7" t="n"/>
       <c r="O11" s="7" t="n"/>
       <c r="P11" s="7" t="n"/>
       <c r="Q11" s="7" t="n"/>
+      <c r="R11" s="7" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="7" t="n"/>
@@ -1756,11 +1831,12 @@
       <c r="J12" s="7" t="n"/>
       <c r="K12" s="7" t="n"/>
       <c r="L12" s="7" t="n"/>
-      <c r="M12" s="7" t="n"/>
+      <c r="M12" s="23" t="n"/>
       <c r="N12" s="7" t="n"/>
       <c r="O12" s="7" t="n"/>
       <c r="P12" s="7" t="n"/>
       <c r="Q12" s="7" t="n"/>
+      <c r="R12" s="7" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="7" t="n"/>
@@ -1775,11 +1851,12 @@
       <c r="J13" s="7" t="n"/>
       <c r="K13" s="7" t="n"/>
       <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7" t="n"/>
+      <c r="M13" s="23" t="n"/>
       <c r="N13" s="7" t="n"/>
       <c r="O13" s="7" t="n"/>
       <c r="P13" s="7" t="n"/>
       <c r="Q13" s="7" t="n"/>
+      <c r="R13" s="7" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="7" t="n"/>
@@ -1794,11 +1871,12 @@
       <c r="J14" s="7" t="n"/>
       <c r="K14" s="7" t="n"/>
       <c r="L14" s="7" t="n"/>
-      <c r="M14" s="7" t="n"/>
+      <c r="M14" s="23" t="n"/>
       <c r="N14" s="7" t="n"/>
       <c r="O14" s="7" t="n"/>
       <c r="P14" s="7" t="n"/>
       <c r="Q14" s="7" t="n"/>
+      <c r="R14" s="7" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="7" t="n"/>
@@ -1813,11 +1891,12 @@
       <c r="J15" s="7" t="n"/>
       <c r="K15" s="7" t="n"/>
       <c r="L15" s="7" t="n"/>
-      <c r="M15" s="7" t="n"/>
+      <c r="M15" s="23" t="n"/>
       <c r="N15" s="7" t="n"/>
       <c r="O15" s="7" t="n"/>
       <c r="P15" s="7" t="n"/>
       <c r="Q15" s="7" t="n"/>
+      <c r="R15" s="7" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="7" t="n"/>
@@ -1832,11 +1911,12 @@
       <c r="J16" s="7" t="n"/>
       <c r="K16" s="7" t="n"/>
       <c r="L16" s="7" t="n"/>
-      <c r="M16" s="7" t="n"/>
+      <c r="M16" s="23" t="n"/>
       <c r="N16" s="7" t="n"/>
       <c r="O16" s="7" t="n"/>
       <c r="P16" s="7" t="n"/>
       <c r="Q16" s="7" t="n"/>
+      <c r="R16" s="7" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="7" t="n"/>
@@ -1851,11 +1931,12 @@
       <c r="J17" s="7" t="n"/>
       <c r="K17" s="7" t="n"/>
       <c r="L17" s="7" t="n"/>
-      <c r="M17" s="7" t="n"/>
+      <c r="M17" s="23" t="n"/>
       <c r="N17" s="7" t="n"/>
       <c r="O17" s="7" t="n"/>
       <c r="P17" s="7" t="n"/>
       <c r="Q17" s="7" t="n"/>
+      <c r="R17" s="7" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="7" t="n"/>
@@ -1870,11 +1951,12 @@
       <c r="J18" s="7" t="n"/>
       <c r="K18" s="7" t="n"/>
       <c r="L18" s="7" t="n"/>
-      <c r="M18" s="7" t="n"/>
+      <c r="M18" s="23" t="n"/>
       <c r="N18" s="7" t="n"/>
       <c r="O18" s="7" t="n"/>
       <c r="P18" s="7" t="n"/>
       <c r="Q18" s="7" t="n"/>
+      <c r="R18" s="7" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="7" t="n"/>
@@ -1889,11 +1971,12 @@
       <c r="J19" s="7" t="n"/>
       <c r="K19" s="7" t="n"/>
       <c r="L19" s="7" t="n"/>
-      <c r="M19" s="7" t="n"/>
+      <c r="M19" s="23" t="n"/>
       <c r="N19" s="7" t="n"/>
       <c r="O19" s="7" t="n"/>
       <c r="P19" s="7" t="n"/>
       <c r="Q19" s="7" t="n"/>
+      <c r="R19" s="7" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="7" t="n"/>
@@ -1908,11 +1991,12 @@
       <c r="J20" s="7" t="n"/>
       <c r="K20" s="7" t="n"/>
       <c r="L20" s="7" t="n"/>
-      <c r="M20" s="7" t="n"/>
+      <c r="M20" s="23" t="n"/>
       <c r="N20" s="7" t="n"/>
       <c r="O20" s="7" t="n"/>
       <c r="P20" s="7" t="n"/>
       <c r="Q20" s="7" t="n"/>
+      <c r="R20" s="7" t="n"/>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
@@ -1931,11 +2015,18 @@
       <c r="J21" s="7" t="n"/>
       <c r="K21" s="7" t="n"/>
       <c r="L21" s="7" t="n"/>
-      <c r="M21" s="7" t="n"/>
+      <c r="M21" s="24">
+        <f>SUM(M8:M20)</f>
+        <v/>
+      </c>
       <c r="N21" s="7" t="n"/>
       <c r="O21" s="7" t="n"/>
       <c r="P21" s="7" t="n"/>
       <c r="Q21" s="7" t="n"/>
+      <c r="R21" s="7" t="n"/>
+    </row>
+    <row r="22">
+      <c r="M22" s="22" t="n"/>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
@@ -1948,26 +2039,29 @@
           <t>SIGNATURE AND SEAL OF HEADMASTER</t>
         </is>
       </c>
+      <c r="M23" s="22" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="20">
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="L23:Q23"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="I3:Q3"/>
+    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="K4:Q4"/>
+    <mergeCell ref="H6:L6"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="F5:J5"/>
+    <mergeCell ref="M6:M7"/>
+    <mergeCell ref="B6:B7"/>
     <mergeCell ref="K5:Q5"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A3:H3"/>
+    <mergeCell ref="M6:Q6"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A4:E4"/>
-    <mergeCell ref="K4:Q4"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="H6:L6"/>
-    <mergeCell ref="M6:Q6"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="F5:J5"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="L23:Q23"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="I3:Q3"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="N6:R6"/>
     <mergeCell ref="F4:J4"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: Add dedicated Arrear Rows under months & fix User Guide modal onclick
</commit_message>
<xml_diff>
--- a/templates/DPO_Muzaffarpur_Arrear_Forms.xlsx
+++ b/templates/DPO_Muzaffarpur_Arrear_Forms.xlsx
@@ -63,21 +63,15 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-        <bgColor rgb="00D9E1F2"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="12">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -197,25 +191,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="00000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="00000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00000000"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -260,17 +240,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -636,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA24"/>
+  <dimension ref="A1:Z24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -654,7 +623,6 @@
     <col width="7" customWidth="1" min="16" max="16"/>
     <col width="6" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="19"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
     <col width="8" customWidth="1" min="20" max="21"/>
     <col width="7" customWidth="1" min="22" max="22"/>
     <col width="10" customWidth="1" min="23" max="23"/>
@@ -704,14 +672,14 @@
       <c r="P3" s="16" t="n"/>
       <c r="Q3" s="16" t="n"/>
       <c r="R3" s="16" t="n"/>
+      <c r="S3" s="16" t="n"/>
       <c r="T3" s="16" t="n"/>
       <c r="U3" s="16" t="n"/>
       <c r="V3" s="16" t="n"/>
       <c r="W3" s="16" t="n"/>
       <c r="X3" s="16" t="n"/>
       <c r="Y3" s="16" t="n"/>
-      <c r="Z3" s="16" t="n"/>
-      <c r="AA3" s="17" t="n"/>
+      <c r="Z3" s="17" t="n"/>
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -744,14 +712,14 @@
         </is>
       </c>
       <c r="R4" s="16" t="n"/>
+      <c r="S4" s="16" t="n"/>
       <c r="T4" s="16" t="n"/>
       <c r="U4" s="16" t="n"/>
       <c r="V4" s="16" t="n"/>
       <c r="W4" s="16" t="n"/>
       <c r="X4" s="16" t="n"/>
       <c r="Y4" s="16" t="n"/>
-      <c r="Z4" s="16" t="n"/>
-      <c r="AA4" s="17" t="n"/>
+      <c r="Z4" s="17" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
@@ -784,14 +752,14 @@
         </is>
       </c>
       <c r="R5" s="16" t="n"/>
+      <c r="S5" s="16" t="n"/>
       <c r="T5" s="16" t="n"/>
       <c r="U5" s="16" t="n"/>
       <c r="V5" s="16" t="n"/>
       <c r="W5" s="16" t="n"/>
       <c r="X5" s="16" t="n"/>
       <c r="Y5" s="16" t="n"/>
-      <c r="Z5" s="16" t="n"/>
-      <c r="AA5" s="17" t="n"/>
+      <c r="Z5" s="17" t="n"/>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
@@ -829,24 +797,18 @@
       <c r="P6" s="16" t="n"/>
       <c r="Q6" s="16" t="n"/>
       <c r="R6" s="17" t="n"/>
-      <c r="S6" s="20" t="inlineStr">
-        <is>
-          <t>PAID
-ARREAR</t>
-        </is>
-      </c>
-      <c r="T6" s="21" t="inlineStr">
+      <c r="S6" s="6" t="inlineStr">
         <is>
           <t>DIFFERENCE</t>
         </is>
       </c>
+      <c r="T6" s="16" t="n"/>
       <c r="U6" s="16" t="n"/>
       <c r="V6" s="16" t="n"/>
       <c r="W6" s="16" t="n"/>
       <c r="X6" s="16" t="n"/>
       <c r="Y6" s="16" t="n"/>
-      <c r="Z6" s="16" t="n"/>
-      <c r="AA6" s="17" t="n"/>
+      <c r="Z6" s="17" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="19" t="n"/>
@@ -937,45 +899,44 @@
 PAY</t>
         </is>
       </c>
-      <c r="S7" s="22" t="n"/>
-      <c r="T7" s="6" t="inlineStr">
+      <c r="S7" s="6" t="inlineStr">
         <is>
           <t>Basic
 Pay</t>
         </is>
       </c>
+      <c r="T7" s="6" t="inlineStr">
+        <is>
+          <t>D.A.</t>
+        </is>
+      </c>
       <c r="U7" s="6" t="inlineStr">
         <is>
-          <t>D.A.</t>
+          <t>H.R.A.</t>
         </is>
       </c>
       <c r="V7" s="6" t="inlineStr">
         <is>
-          <t>H.R.A.</t>
+          <t>M.A.</t>
         </is>
       </c>
       <c r="W7" s="6" t="inlineStr">
-        <is>
-          <t>M.A.</t>
-        </is>
-      </c>
-      <c r="X7" s="6" t="inlineStr">
         <is>
           <t>GROSS
 PAY</t>
         </is>
       </c>
+      <c r="X7" s="6" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
       <c r="Y7" s="6" t="inlineStr">
         <is>
-          <t>NPS</t>
+          <t>GIS</t>
         </is>
       </c>
       <c r="Z7" s="6" t="inlineStr">
-        <is>
-          <t>GIS</t>
-        </is>
-      </c>
-      <c r="AA7" s="6" t="inlineStr">
         <is>
           <t>NET
 PAY</t>
@@ -1001,7 +962,7 @@
       <c r="P8" s="7" t="n"/>
       <c r="Q8" s="7" t="n"/>
       <c r="R8" s="7" t="n"/>
-      <c r="S8" s="23" t="n"/>
+      <c r="S8" s="7" t="n"/>
       <c r="T8" s="7" t="n"/>
       <c r="U8" s="7" t="n"/>
       <c r="V8" s="7" t="n"/>
@@ -1009,7 +970,6 @@
       <c r="X8" s="7" t="n"/>
       <c r="Y8" s="7" t="n"/>
       <c r="Z8" s="7" t="n"/>
-      <c r="AA8" s="7" t="n"/>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="7" t="n"/>
@@ -1030,7 +990,7 @@
       <c r="P9" s="7" t="n"/>
       <c r="Q9" s="7" t="n"/>
       <c r="R9" s="7" t="n"/>
-      <c r="S9" s="23" t="n"/>
+      <c r="S9" s="7" t="n"/>
       <c r="T9" s="7" t="n"/>
       <c r="U9" s="7" t="n"/>
       <c r="V9" s="7" t="n"/>
@@ -1038,7 +998,6 @@
       <c r="X9" s="7" t="n"/>
       <c r="Y9" s="7" t="n"/>
       <c r="Z9" s="7" t="n"/>
-      <c r="AA9" s="7" t="n"/>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="7" t="n"/>
@@ -1059,7 +1018,7 @@
       <c r="P10" s="7" t="n"/>
       <c r="Q10" s="7" t="n"/>
       <c r="R10" s="7" t="n"/>
-      <c r="S10" s="23" t="n"/>
+      <c r="S10" s="7" t="n"/>
       <c r="T10" s="7" t="n"/>
       <c r="U10" s="7" t="n"/>
       <c r="V10" s="7" t="n"/>
@@ -1067,7 +1026,6 @@
       <c r="X10" s="7" t="n"/>
       <c r="Y10" s="7" t="n"/>
       <c r="Z10" s="7" t="n"/>
-      <c r="AA10" s="7" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="7" t="n"/>
@@ -1088,7 +1046,7 @@
       <c r="P11" s="7" t="n"/>
       <c r="Q11" s="7" t="n"/>
       <c r="R11" s="7" t="n"/>
-      <c r="S11" s="23" t="n"/>
+      <c r="S11" s="7" t="n"/>
       <c r="T11" s="7" t="n"/>
       <c r="U11" s="7" t="n"/>
       <c r="V11" s="7" t="n"/>
@@ -1096,7 +1054,6 @@
       <c r="X11" s="7" t="n"/>
       <c r="Y11" s="7" t="n"/>
       <c r="Z11" s="7" t="n"/>
-      <c r="AA11" s="7" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="7" t="n"/>
@@ -1117,7 +1074,7 @@
       <c r="P12" s="7" t="n"/>
       <c r="Q12" s="7" t="n"/>
       <c r="R12" s="7" t="n"/>
-      <c r="S12" s="23" t="n"/>
+      <c r="S12" s="7" t="n"/>
       <c r="T12" s="7" t="n"/>
       <c r="U12" s="7" t="n"/>
       <c r="V12" s="7" t="n"/>
@@ -1125,7 +1082,6 @@
       <c r="X12" s="7" t="n"/>
       <c r="Y12" s="7" t="n"/>
       <c r="Z12" s="7" t="n"/>
-      <c r="AA12" s="7" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="7" t="n"/>
@@ -1146,7 +1102,7 @@
       <c r="P13" s="7" t="n"/>
       <c r="Q13" s="7" t="n"/>
       <c r="R13" s="7" t="n"/>
-      <c r="S13" s="23" t="n"/>
+      <c r="S13" s="7" t="n"/>
       <c r="T13" s="7" t="n"/>
       <c r="U13" s="7" t="n"/>
       <c r="V13" s="7" t="n"/>
@@ -1154,7 +1110,6 @@
       <c r="X13" s="7" t="n"/>
       <c r="Y13" s="7" t="n"/>
       <c r="Z13" s="7" t="n"/>
-      <c r="AA13" s="7" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="7" t="n"/>
@@ -1175,7 +1130,7 @@
       <c r="P14" s="7" t="n"/>
       <c r="Q14" s="7" t="n"/>
       <c r="R14" s="7" t="n"/>
-      <c r="S14" s="23" t="n"/>
+      <c r="S14" s="7" t="n"/>
       <c r="T14" s="7" t="n"/>
       <c r="U14" s="7" t="n"/>
       <c r="V14" s="7" t="n"/>
@@ -1183,7 +1138,6 @@
       <c r="X14" s="7" t="n"/>
       <c r="Y14" s="7" t="n"/>
       <c r="Z14" s="7" t="n"/>
-      <c r="AA14" s="7" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="7" t="n"/>
@@ -1204,7 +1158,7 @@
       <c r="P15" s="7" t="n"/>
       <c r="Q15" s="7" t="n"/>
       <c r="R15" s="7" t="n"/>
-      <c r="S15" s="23" t="n"/>
+      <c r="S15" s="7" t="n"/>
       <c r="T15" s="7" t="n"/>
       <c r="U15" s="7" t="n"/>
       <c r="V15" s="7" t="n"/>
@@ -1212,7 +1166,6 @@
       <c r="X15" s="7" t="n"/>
       <c r="Y15" s="7" t="n"/>
       <c r="Z15" s="7" t="n"/>
-      <c r="AA15" s="7" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="7" t="n"/>
@@ -1233,7 +1186,7 @@
       <c r="P16" s="7" t="n"/>
       <c r="Q16" s="7" t="n"/>
       <c r="R16" s="7" t="n"/>
-      <c r="S16" s="23" t="n"/>
+      <c r="S16" s="7" t="n"/>
       <c r="T16" s="7" t="n"/>
       <c r="U16" s="7" t="n"/>
       <c r="V16" s="7" t="n"/>
@@ -1241,7 +1194,6 @@
       <c r="X16" s="7" t="n"/>
       <c r="Y16" s="7" t="n"/>
       <c r="Z16" s="7" t="n"/>
-      <c r="AA16" s="7" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="7" t="n"/>
@@ -1262,7 +1214,7 @@
       <c r="P17" s="7" t="n"/>
       <c r="Q17" s="7" t="n"/>
       <c r="R17" s="7" t="n"/>
-      <c r="S17" s="23" t="n"/>
+      <c r="S17" s="7" t="n"/>
       <c r="T17" s="7" t="n"/>
       <c r="U17" s="7" t="n"/>
       <c r="V17" s="7" t="n"/>
@@ -1270,7 +1222,6 @@
       <c r="X17" s="7" t="n"/>
       <c r="Y17" s="7" t="n"/>
       <c r="Z17" s="7" t="n"/>
-      <c r="AA17" s="7" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="7" t="n"/>
@@ -1291,7 +1242,7 @@
       <c r="P18" s="7" t="n"/>
       <c r="Q18" s="7" t="n"/>
       <c r="R18" s="7" t="n"/>
-      <c r="S18" s="23" t="n"/>
+      <c r="S18" s="7" t="n"/>
       <c r="T18" s="7" t="n"/>
       <c r="U18" s="7" t="n"/>
       <c r="V18" s="7" t="n"/>
@@ -1299,7 +1250,6 @@
       <c r="X18" s="7" t="n"/>
       <c r="Y18" s="7" t="n"/>
       <c r="Z18" s="7" t="n"/>
-      <c r="AA18" s="7" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="7" t="n"/>
@@ -1320,7 +1270,7 @@
       <c r="P19" s="7" t="n"/>
       <c r="Q19" s="7" t="n"/>
       <c r="R19" s="7" t="n"/>
-      <c r="S19" s="23" t="n"/>
+      <c r="S19" s="7" t="n"/>
       <c r="T19" s="7" t="n"/>
       <c r="U19" s="7" t="n"/>
       <c r="V19" s="7" t="n"/>
@@ -1328,7 +1278,6 @@
       <c r="X19" s="7" t="n"/>
       <c r="Y19" s="7" t="n"/>
       <c r="Z19" s="7" t="n"/>
-      <c r="AA19" s="7" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="7" t="n"/>
@@ -1349,7 +1298,7 @@
       <c r="P20" s="7" t="n"/>
       <c r="Q20" s="7" t="n"/>
       <c r="R20" s="7" t="n"/>
-      <c r="S20" s="23" t="n"/>
+      <c r="S20" s="7" t="n"/>
       <c r="T20" s="7" t="n"/>
       <c r="U20" s="7" t="n"/>
       <c r="V20" s="7" t="n"/>
@@ -1357,7 +1306,6 @@
       <c r="X20" s="7" t="n"/>
       <c r="Y20" s="7" t="n"/>
       <c r="Z20" s="7" t="n"/>
-      <c r="AA20" s="7" t="n"/>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
@@ -1382,10 +1330,7 @@
       <c r="P21" s="7" t="n"/>
       <c r="Q21" s="7" t="n"/>
       <c r="R21" s="7" t="n"/>
-      <c r="S21" s="24">
-        <f>SUM(S8:S20)</f>
-        <v/>
-      </c>
+      <c r="S21" s="7" t="n"/>
       <c r="T21" s="7" t="n"/>
       <c r="U21" s="7" t="n"/>
       <c r="V21" s="7" t="n"/>
@@ -1393,7 +1338,6 @@
       <c r="X21" s="7" t="n"/>
       <c r="Y21" s="7" t="n"/>
       <c r="Z21" s="7" t="n"/>
-      <c r="AA21" s="7" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="3" t="n"/>
@@ -1418,18 +1362,14 @@
       <c r="P22" s="16" t="n"/>
       <c r="Q22" s="16" t="n"/>
       <c r="R22" s="16" t="n"/>
-      <c r="S22" s="22" t="n"/>
+      <c r="S22" s="16" t="n"/>
       <c r="T22" s="16" t="n"/>
       <c r="U22" s="16" t="n"/>
       <c r="V22" s="16" t="n"/>
       <c r="W22" s="16" t="n"/>
       <c r="X22" s="16" t="n"/>
       <c r="Y22" s="16" t="n"/>
-      <c r="Z22" s="16" t="n"/>
-      <c r="AA22" s="17" t="n"/>
-    </row>
-    <row r="23">
-      <c r="S23" s="22" t="n"/>
+      <c r="Z22" s="17" t="n"/>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
@@ -1442,17 +1382,15 @@
           <t>SIGNATURE AND SEAL OF HEADMASTER</t>
         </is>
       </c>
-      <c r="S24" s="22" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="19">
     <mergeCell ref="R24:Z24"/>
     <mergeCell ref="C6:J6"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="C22:Z22"/>
     <mergeCell ref="A1:Z1"/>
     <mergeCell ref="B6:B7"/>
-    <mergeCell ref="S6:S7"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="S6:Z6"/>
     <mergeCell ref="N3:Z3"/>
@@ -1464,7 +1402,6 @@
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="I4:P4"/>
     <mergeCell ref="Q4:Z4"/>
-    <mergeCell ref="T6:AA6"/>
     <mergeCell ref="A3:M3"/>
     <mergeCell ref="K6:R6"/>
   </mergeCells>
@@ -1479,7 +1416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R23"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1493,7 +1430,6 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="13"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="8" customWidth="1" min="16" max="16"/>
@@ -1535,11 +1471,11 @@
       <c r="J3" s="16" t="n"/>
       <c r="K3" s="16" t="n"/>
       <c r="L3" s="16" t="n"/>
+      <c r="M3" s="16" t="n"/>
       <c r="N3" s="16" t="n"/>
       <c r="O3" s="16" t="n"/>
       <c r="P3" s="16" t="n"/>
-      <c r="Q3" s="16" t="n"/>
-      <c r="R3" s="17" t="n"/>
+      <c r="Q3" s="17" t="n"/>
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -1566,11 +1502,11 @@
         </is>
       </c>
       <c r="L4" s="16" t="n"/>
+      <c r="M4" s="16" t="n"/>
       <c r="N4" s="16" t="n"/>
       <c r="O4" s="16" t="n"/>
       <c r="P4" s="16" t="n"/>
-      <c r="Q4" s="16" t="n"/>
-      <c r="R4" s="17" t="n"/>
+      <c r="Q4" s="17" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
@@ -1597,11 +1533,11 @@
         </is>
       </c>
       <c r="L5" s="16" t="n"/>
+      <c r="M5" s="16" t="n"/>
       <c r="N5" s="16" t="n"/>
       <c r="O5" s="16" t="n"/>
       <c r="P5" s="16" t="n"/>
-      <c r="Q5" s="16" t="n"/>
-      <c r="R5" s="17" t="n"/>
+      <c r="Q5" s="17" t="n"/>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
@@ -1633,21 +1569,15 @@
       <c r="J6" s="16" t="n"/>
       <c r="K6" s="16" t="n"/>
       <c r="L6" s="17" t="n"/>
-      <c r="M6" s="20" t="inlineStr">
-        <is>
-          <t>PAID
-ARREAR</t>
-        </is>
-      </c>
-      <c r="N6" s="21" t="inlineStr">
+      <c r="M6" s="6" t="inlineStr">
         <is>
           <t>DIFFERENCE</t>
         </is>
       </c>
+      <c r="N6" s="16" t="n"/>
       <c r="O6" s="16" t="n"/>
       <c r="P6" s="16" t="n"/>
-      <c r="Q6" s="16" t="n"/>
-      <c r="R6" s="17" t="n"/>
+      <c r="Q6" s="17" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="19" t="n"/>
@@ -1708,30 +1638,29 @@
 AMOUNT</t>
         </is>
       </c>
-      <c r="M7" s="22" t="n"/>
-      <c r="N7" s="6" t="inlineStr">
+      <c r="M7" s="6" t="inlineStr">
         <is>
           <t>Basic
 Pay</t>
         </is>
       </c>
+      <c r="N7" s="6" t="inlineStr">
+        <is>
+          <t>D.A.</t>
+        </is>
+      </c>
       <c r="O7" s="6" t="inlineStr">
-        <is>
-          <t>D.A.</t>
-        </is>
-      </c>
-      <c r="P7" s="6" t="inlineStr">
         <is>
           <t>GROSS
 AMOUNT</t>
         </is>
       </c>
+      <c r="P7" s="6" t="inlineStr">
+        <is>
+          <t>NPS</t>
+        </is>
+      </c>
       <c r="Q7" s="6" t="inlineStr">
-        <is>
-          <t>NPS</t>
-        </is>
-      </c>
-      <c r="R7" s="6" t="inlineStr">
         <is>
           <t>NET
 AMOUNT</t>
@@ -1751,12 +1680,11 @@
       <c r="J8" s="7" t="n"/>
       <c r="K8" s="7" t="n"/>
       <c r="L8" s="7" t="n"/>
-      <c r="M8" s="23" t="n"/>
+      <c r="M8" s="7" t="n"/>
       <c r="N8" s="7" t="n"/>
       <c r="O8" s="7" t="n"/>
       <c r="P8" s="7" t="n"/>
       <c r="Q8" s="7" t="n"/>
-      <c r="R8" s="7" t="n"/>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="7" t="n"/>
@@ -1771,12 +1699,11 @@
       <c r="J9" s="7" t="n"/>
       <c r="K9" s="7" t="n"/>
       <c r="L9" s="7" t="n"/>
-      <c r="M9" s="23" t="n"/>
+      <c r="M9" s="7" t="n"/>
       <c r="N9" s="7" t="n"/>
       <c r="O9" s="7" t="n"/>
       <c r="P9" s="7" t="n"/>
       <c r="Q9" s="7" t="n"/>
-      <c r="R9" s="7" t="n"/>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="7" t="n"/>
@@ -1791,12 +1718,11 @@
       <c r="J10" s="7" t="n"/>
       <c r="K10" s="7" t="n"/>
       <c r="L10" s="7" t="n"/>
-      <c r="M10" s="23" t="n"/>
+      <c r="M10" s="7" t="n"/>
       <c r="N10" s="7" t="n"/>
       <c r="O10" s="7" t="n"/>
       <c r="P10" s="7" t="n"/>
       <c r="Q10" s="7" t="n"/>
-      <c r="R10" s="7" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="7" t="n"/>
@@ -1811,12 +1737,11 @@
       <c r="J11" s="7" t="n"/>
       <c r="K11" s="7" t="n"/>
       <c r="L11" s="7" t="n"/>
-      <c r="M11" s="23" t="n"/>
+      <c r="M11" s="7" t="n"/>
       <c r="N11" s="7" t="n"/>
       <c r="O11" s="7" t="n"/>
       <c r="P11" s="7" t="n"/>
       <c r="Q11" s="7" t="n"/>
-      <c r="R11" s="7" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="7" t="n"/>
@@ -1831,12 +1756,11 @@
       <c r="J12" s="7" t="n"/>
       <c r="K12" s="7" t="n"/>
       <c r="L12" s="7" t="n"/>
-      <c r="M12" s="23" t="n"/>
+      <c r="M12" s="7" t="n"/>
       <c r="N12" s="7" t="n"/>
       <c r="O12" s="7" t="n"/>
       <c r="P12" s="7" t="n"/>
       <c r="Q12" s="7" t="n"/>
-      <c r="R12" s="7" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="7" t="n"/>
@@ -1851,12 +1775,11 @@
       <c r="J13" s="7" t="n"/>
       <c r="K13" s="7" t="n"/>
       <c r="L13" s="7" t="n"/>
-      <c r="M13" s="23" t="n"/>
+      <c r="M13" s="7" t="n"/>
       <c r="N13" s="7" t="n"/>
       <c r="O13" s="7" t="n"/>
       <c r="P13" s="7" t="n"/>
       <c r="Q13" s="7" t="n"/>
-      <c r="R13" s="7" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="7" t="n"/>
@@ -1871,12 +1794,11 @@
       <c r="J14" s="7" t="n"/>
       <c r="K14" s="7" t="n"/>
       <c r="L14" s="7" t="n"/>
-      <c r="M14" s="23" t="n"/>
+      <c r="M14" s="7" t="n"/>
       <c r="N14" s="7" t="n"/>
       <c r="O14" s="7" t="n"/>
       <c r="P14" s="7" t="n"/>
       <c r="Q14" s="7" t="n"/>
-      <c r="R14" s="7" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="7" t="n"/>
@@ -1891,12 +1813,11 @@
       <c r="J15" s="7" t="n"/>
       <c r="K15" s="7" t="n"/>
       <c r="L15" s="7" t="n"/>
-      <c r="M15" s="23" t="n"/>
+      <c r="M15" s="7" t="n"/>
       <c r="N15" s="7" t="n"/>
       <c r="O15" s="7" t="n"/>
       <c r="P15" s="7" t="n"/>
       <c r="Q15" s="7" t="n"/>
-      <c r="R15" s="7" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="7" t="n"/>
@@ -1911,12 +1832,11 @@
       <c r="J16" s="7" t="n"/>
       <c r="K16" s="7" t="n"/>
       <c r="L16" s="7" t="n"/>
-      <c r="M16" s="23" t="n"/>
+      <c r="M16" s="7" t="n"/>
       <c r="N16" s="7" t="n"/>
       <c r="O16" s="7" t="n"/>
       <c r="P16" s="7" t="n"/>
       <c r="Q16" s="7" t="n"/>
-      <c r="R16" s="7" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="7" t="n"/>
@@ -1931,12 +1851,11 @@
       <c r="J17" s="7" t="n"/>
       <c r="K17" s="7" t="n"/>
       <c r="L17" s="7" t="n"/>
-      <c r="M17" s="23" t="n"/>
+      <c r="M17" s="7" t="n"/>
       <c r="N17" s="7" t="n"/>
       <c r="O17" s="7" t="n"/>
       <c r="P17" s="7" t="n"/>
       <c r="Q17" s="7" t="n"/>
-      <c r="R17" s="7" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="7" t="n"/>
@@ -1951,12 +1870,11 @@
       <c r="J18" s="7" t="n"/>
       <c r="K18" s="7" t="n"/>
       <c r="L18" s="7" t="n"/>
-      <c r="M18" s="23" t="n"/>
+      <c r="M18" s="7" t="n"/>
       <c r="N18" s="7" t="n"/>
       <c r="O18" s="7" t="n"/>
       <c r="P18" s="7" t="n"/>
       <c r="Q18" s="7" t="n"/>
-      <c r="R18" s="7" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="7" t="n"/>
@@ -1971,12 +1889,11 @@
       <c r="J19" s="7" t="n"/>
       <c r="K19" s="7" t="n"/>
       <c r="L19" s="7" t="n"/>
-      <c r="M19" s="23" t="n"/>
+      <c r="M19" s="7" t="n"/>
       <c r="N19" s="7" t="n"/>
       <c r="O19" s="7" t="n"/>
       <c r="P19" s="7" t="n"/>
       <c r="Q19" s="7" t="n"/>
-      <c r="R19" s="7" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="7" t="n"/>
@@ -1991,12 +1908,11 @@
       <c r="J20" s="7" t="n"/>
       <c r="K20" s="7" t="n"/>
       <c r="L20" s="7" t="n"/>
-      <c r="M20" s="23" t="n"/>
+      <c r="M20" s="7" t="n"/>
       <c r="N20" s="7" t="n"/>
       <c r="O20" s="7" t="n"/>
       <c r="P20" s="7" t="n"/>
       <c r="Q20" s="7" t="n"/>
-      <c r="R20" s="7" t="n"/>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
@@ -2015,18 +1931,11 @@
       <c r="J21" s="7" t="n"/>
       <c r="K21" s="7" t="n"/>
       <c r="L21" s="7" t="n"/>
-      <c r="M21" s="24">
-        <f>SUM(M8:M20)</f>
-        <v/>
-      </c>
+      <c r="M21" s="7" t="n"/>
       <c r="N21" s="7" t="n"/>
       <c r="O21" s="7" t="n"/>
       <c r="P21" s="7" t="n"/>
       <c r="Q21" s="7" t="n"/>
-      <c r="R21" s="7" t="n"/>
-    </row>
-    <row r="22">
-      <c r="M22" s="22" t="n"/>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
@@ -2039,29 +1948,26 @@
           <t>SIGNATURE AND SEAL OF HEADMASTER</t>
         </is>
       </c>
-      <c r="M23" s="22" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="18">
+    <mergeCell ref="K5:Q5"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="K4:Q4"/>
     <mergeCell ref="C6:G6"/>
+    <mergeCell ref="H6:L6"/>
+    <mergeCell ref="M6:Q6"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="F5:J5"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="L23:Q23"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="I3:Q3"/>
+    <mergeCell ref="B6:B7"/>
     <mergeCell ref="A1:Q1"/>
-    <mergeCell ref="K4:Q4"/>
-    <mergeCell ref="H6:L6"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="F5:J5"/>
-    <mergeCell ref="M6:M7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="K5:Q5"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="M6:Q6"/>
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="N6:R6"/>
     <mergeCell ref="F4:J4"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>

</xml_diff>